<commit_message>
Budget v0.2 for merged programme (4 nights, goûter, maquis, Grand-Bassam, KAVA)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsKwZ4mhRTGki8ZCbBAtxZ
</commit_message>
<xml_diff>
--- a/03-budget/ground-budget.xlsx
+++ b/03-budget/ground-budget.xlsx
@@ -534,11 +534,11 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nights of 19, 20, 21 Oct; depart 22 Oct to Monrovia</t>
+          <t>Nights of 18–21 Oct (arrive the evening before); depart 22 Oct to Monrovia</t>
         </is>
       </c>
     </row>
@@ -564,11 +564,11 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Arrival day through airport drop on 22 Oct</t>
+          <t>18 Oct airport pick-up through 22 Oct airport drop</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -661,7 +661,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chef Abbys × Côte d'Ivoire · 19–21 Oct 2026 · Ground budget (pre-quote estimate)</t>
+          <t>Chef Abbys × Côte d'Ivoire · 19–21 Oct 2026 · Ground budget v0.2 (pre-quote estimate)</t>
         </is>
       </c>
     </row>
@@ -754,14 +754,10 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>In-kind: airport / ministry protocol</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Ministry of Tourism protocol may cover</t>
-        </is>
-      </c>
+          <t>In-kind: ministry protocol</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -771,7 +767,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Hotel 4–5★ Abidjan, single rooms</t>
+          <t>L'Avenue Hôtel (or equivalent), single rooms</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
@@ -806,7 +802,7 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Target: Sofitel Hôtel Ivoire / Noom / Pullman</t>
+          <t>Rate to quote</t>
         </is>
       </c>
     </row>
@@ -825,7 +821,7 @@
         <v>25000</v>
       </c>
       <c r="D5" s="6">
-        <f>Assumptions!$B$3*Assumptions!$B$5</f>
+        <f>Assumptions!$B$3*Assumptions!$B$4</f>
         <v/>
       </c>
       <c r="E5" s="7">
@@ -941,11 +937,7 @@
           <t>In-kind: mobility partner</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>inDrive / Yango / dealer</t>
-        </is>
-      </c>
+      <c r="J7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -998,11 +990,11 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Fuel &amp; tolls supplement — Dabou / Jacqueville run</t>
+          <t>Fuel &amp; tolls supplement — Grand-Bassam run</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>60000</v>
+        <v>40000</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>1</v>
@@ -1030,11 +1022,7 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>~2 × 60 km + bridge</t>
-        </is>
-      </c>
+      <c r="J9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -1172,16 +1160,16 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · The Bean</t>
+          <t>Day 1 · The lagoon</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Private bean-to-bar workshop — Le Chocolatier Ivoirien</t>
+          <t>Attiéké entrepreneur — workshop honorarium</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>500000</v>
+        <v>300000</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>1</v>
@@ -1206,32 +1194,31 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>In-kind / co-brand</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Axel-Emmanuel Gbaou, Cocody</t>
+          <t>Women-led brand, to identify</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · The Bean</t>
+          <t>Day 1 · The lagoon</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Welcome dinner with a leading Ivorian chef (party + ~8 guests)</t>
+          <t>Lagoon beach location, set &amp; access</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>45000</v>
-      </c>
-      <c r="D14" s="6">
-        <f>Assumptions!$B$3+8</f>
-        <v/>
+        <v>150000</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="E14" s="7">
         <f>IF(H14="Y",C14*D14,0)</f>
@@ -1253,28 +1240,28 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>e.g. Charlie Koffi, Villa Alfira</t>
+          <t>Site to confirm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · The Lagoon</t>
+          <t>Day 1 · The lagoon</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Honorarium — Attiéké des Lagunes women's group (Dabou)</t>
+          <t>Garba ingredients &amp; tasting</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>300000</v>
+        <v>60000</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>
@@ -1302,28 +1289,24 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>Direct to the cooperative</t>
-        </is>
-      </c>
+      <c r="J15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · The Lagoon</t>
+          <t>Day 1 · Snack time</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Customary protocol — chiefs, drinks, gifts (2 villages)</t>
+          <t>Goûter ingredients &amp; kit (~40 children)</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="7">
         <f>IF(H16="Y",C16*D16,0)</f>
@@ -1345,31 +1328,31 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Non-negotiable courtesy</t>
+          <t>With Fondation Olivia Yacé</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · The Lagoon</t>
+          <t>Day 1 · Snack time</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>School lunch — meals for pupils</t>
+          <t>Burners, gas, aprons, hygiene</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>1500</v>
+        <v>150000</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="E17" s="7">
         <f>IF(H17="Y",C17*D17,0)</f>
@@ -1391,28 +1374,24 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>~400 pupils; scale to school size</t>
-        </is>
-      </c>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · The Lagoon</t>
+          <t>Day 1 · Snack time</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Outdoor kitchen: tent, burners, gas, chairs, utensils</t>
+          <t>Child-safeguarding officer + consent forms</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>250000</v>
+        <v>100000</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>1</v>
@@ -1442,19 +1421,19 @@
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Rain cover — short rainy season</t>
+          <t>Non-negotiable</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · The Lagoon</t>
+          <t>Day 1 · Maquis night</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Maquis night: reserved space + live band</t>
+          <t>Reserved space + live band</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
@@ -1486,21 +1465,17 @@
           <t>Sponsor</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>Yopougon / Marcory</t>
-        </is>
-      </c>
+      <c r="J19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · The Lagoon</t>
+          <t>Day 1 · Maquis night</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Maquis night: food &amp; drinks (party + ~6 locals)</t>
+          <t>Food &amp; drinks (party + ~6 guests)</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
@@ -1538,16 +1513,16 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · The Table</t>
+          <t>Day 1 · Maquis night</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Musée des Civilisations — guided private visit</t>
+          <t>Jiaan Wu — co-host fee [TBC]</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>50000</v>
+        <v>300000</v>
       </c>
       <c r="D21" s="6" t="n">
         <v>1</v>
@@ -1572,24 +1547,28 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>In-kind: Ministry of Culture</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr"/>
+          <t>Paid / exposure swap</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>Placeholder until quoted</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · The Table</t>
+          <t>Day 2 · Grand-Bassam</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Cook-off venue (lagoon terrace / villa)</t>
+          <t>Zeinab Bancé — foutou workshop fee</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>600000</v>
+        <v>500000</v>
       </c>
       <c r="D22" s="6" t="n">
         <v>1</v>
@@ -1614,24 +1593,28 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>In-kind: venue</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr"/>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>Placeholder until quoted</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · The Table</t>
+          <t>Day 2 · Grand-Bassam</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Cook-off ingredients</t>
+          <t>Lagoon-side garden location</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="D23" s="6" t="n">
         <v>1</v>
@@ -1656,7 +1639,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>In-kind: venue</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr"/>
@@ -1664,16 +1647,16 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · The Table</t>
+          <t>Day 2 · Grand-Bassam</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Cook-off set dressing &amp; kitchen equipment</t>
+          <t>Ingredients, mortar, artisan crockery</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>300000</v>
+        <v>150000</v>
       </c>
       <c r="D24" s="6" t="n">
         <v>1</v>
@@ -1706,19 +1689,19 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · The Table</t>
+          <t>Day 2 · Grand-Bassam</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>FCI 2026 laureates — honoraria (×2)</t>
+          <t>Heritage-quarter guide</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>150000</v>
+        <v>50000</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="7">
         <f>IF(H25="Y",C25*D25,0)</f>
@@ -1740,28 +1723,24 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>In-kind: Ministry of Tourism</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>Festival de la Cuisine Ivoirienne winners</t>
-        </is>
-      </c>
+          <t>In-kind: Ministry of Culture</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · The Table</t>
+          <t>Day 3 · Cocoa &amp; zaouli</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Courtesy-call gifts (ministry / foundation)</t>
+          <t>Maison Mandjou atelier (Ahoua Touré)</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>100000</v>
+        <v>400000</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>1</v>
@@ -1786,7 +1765,7 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>In-kind / co-brand</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr"/>
@@ -1794,19 +1773,19 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Production support</t>
+          <t>Day 3 · Cocoa &amp; zaouli</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Licensed drone operator + ANAC authorisation</t>
+          <t>Bean-to-bar demo — partner chocolatier</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>350000</v>
+        <v>300000</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="7">
         <f>IF(H27="Y",C27*D27,0)</f>
@@ -1828,32 +1807,31 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>In-kind / co-brand</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>Days 2 &amp; 3</t>
+          <t>e.g. Le Chocolatier Ivoirien</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Production support</t>
+          <t>Day 3 · Cocoa &amp; zaouli</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Welcome kit — pagne, AToure merch</t>
+          <t>Gouro zaouli troupe + musicians at KAVA</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D28" s="6">
-        <f>Assumptions!$B$3</f>
-        <v/>
+        <v>600000</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="E28" s="7">
         <f>IF(H28="Y",C28*D28,0)</f>
@@ -1875,255 +1853,247 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
+          <t>In-kind: Ministry of Culture</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Day 3 · Cocoa &amp; zaouli</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Customary gifts &amp; drinks — troupe</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="7">
+        <f>IF(H29="Y",C29*D29,0)</f>
+        <v/>
+      </c>
+      <c r="F29" s="8">
+        <f>E29/Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Ivorian food creators — collab fees (×3)</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D29" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E29" s="11">
-        <f>IF(H29="Y",C29*D29,0)</f>
-        <v/>
-      </c>
-      <c r="F29" s="12">
-        <f>E29/Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="G29" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I29" s="10" t="inlineStr">
-        <is>
-          <t>Often exposure-for-exposure</t>
-        </is>
-      </c>
-      <c r="J29" s="10" t="inlineStr">
-        <is>
-          <t>e.g. @afrofoodie, Ebenezer, Prince Edja</t>
-        </is>
-      </c>
+      <c r="J29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>School donation — kitchen equipment &amp; books</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="n">
-        <v>500000</v>
-      </c>
-      <c r="D30" s="10" t="n">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Day 3 · Closing table</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Closing dinner (party + ~10 guests)</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D30" s="6">
+        <f>Assumptions!$B$3+10</f>
+        <v/>
+      </c>
+      <c r="E30" s="7">
+        <f>IF(H30="Y",C30*D30,0)</f>
+        <v/>
+      </c>
+      <c r="F30" s="8">
+        <f>E30/Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>Ministers, Olivia, chefs</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Day 3 · Closing table</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Courtesy gifts (ministries, foundation)</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D31" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="11">
-        <f>IF(H30="Y",C30*D30,0)</f>
-        <v/>
-      </c>
-      <c r="F30" s="12">
-        <f>E30/Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H30" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I30" s="10" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
-      <c r="J30" s="10" t="inlineStr">
-        <is>
-          <t>Leaves something behind</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Sunset lagoon pinasse — farewell</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="n">
-        <v>400000</v>
-      </c>
-      <c r="D31" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="11">
+      <c r="E31" s="7">
         <f>IF(H31="Y",C31*D31,0)</f>
         <v/>
       </c>
-      <c r="F31" s="12">
+      <c r="F31" s="8">
         <f>E31/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G31" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H31" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I31" s="10" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
-      <c r="J31" s="10" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Local BTS photographer / videographer (sponsor assets)</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D32" s="10">
-        <f>Assumptions!$B$5</f>
-        <v/>
-      </c>
-      <c r="E32" s="11">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Production support</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Licensed drone operator + ANAC authorisation</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>350000</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="7">
         <f>IF(H32="Y",C32*D32,0)</f>
         <v/>
       </c>
-      <c r="F32" s="12">
+      <c r="F32" s="8">
         <f>E32/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G32" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H32" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I32" s="10" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="J32" s="10" t="inlineStr">
-        <is>
-          <t>Deliverables for sponsors &amp; ministry</t>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>Days 1 &amp; 2</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Cocoa farm visit — Azaguié / Abbé-Bégnini (half day)</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="11">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Production support</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Welcome kit — pagne, AToure merch</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D33" s="6">
+        <f>Assumptions!$B$3</f>
+        <v/>
+      </c>
+      <c r="E33" s="7">
         <f>IF(H33="Y",C33*D33,0)</f>
         <v/>
       </c>
-      <c r="F33" s="12">
+      <c r="F33" s="8">
         <f>E33/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G33" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H33" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I33" s="10" t="inlineStr">
-        <is>
-          <t>In-kind: Conseil Café-Cacao</t>
-        </is>
-      </c>
-      <c r="J33" s="10" t="inlineStr">
-        <is>
-          <t>Replaces Day 1 AM free block</t>
-        </is>
-      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Travel (outside ground)</t>
+          <t>Upgrades</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Flights Accra → Abidjan</t>
+          <t>CASOF × Abidjan masterclass (20–30 young cooks)</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D34" s="10">
-        <f>Assumptions!$B$3</f>
-        <v/>
+        <v>300000</v>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E34" s="11">
         <f>IF(H34="Y",C34*D34,0)</f>
@@ -2135,7 +2105,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr">
@@ -2145,32 +2115,27 @@
       </c>
       <c r="I34" s="10" t="inlineStr">
         <is>
-          <t>In-kind: airline</t>
-        </is>
-      </c>
-      <c r="J34" s="10" t="inlineStr">
-        <is>
-          <t>May be on tour budget already</t>
-        </is>
-      </c>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="J34" s="10" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Travel (outside ground)</t>
+          <t>Upgrades</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Flights Abidjan → Monrovia (Air Côte d'Ivoire)</t>
+          <t>Cocoa farm visit (half day)</t>
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>280000</v>
-      </c>
-      <c r="D35" s="10">
-        <f>Assumptions!$B$3</f>
-        <v/>
+        <v>300000</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E35" s="11">
         <f>IF(H35="Y",C35*D35,0)</f>
@@ -2182,7 +2147,7 @@
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="H35" s="13" t="inlineStr">
@@ -2192,31 +2157,27 @@
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>In-kind: Air Côte d'Ivoire</t>
-        </is>
-      </c>
-      <c r="J35" s="10" t="inlineStr">
-        <is>
-          <t>Check days for 22 Oct</t>
-        </is>
-      </c>
+          <t>In-kind: Conseil Café-Cacao</t>
+        </is>
+      </c>
+      <c r="J35" s="10" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Travel (outside ground)</t>
+          <t>Upgrades</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>E-visas for non-ECOWAS crew</t>
+          <t>Sunset pinasse on the Ébrié lagoon</t>
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>50000</v>
+        <v>400000</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" s="11">
         <f>IF(H36="Y",C36*D36,0)</f>
@@ -2228,93 +2189,262 @@
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I36" s="10" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="J36" s="10" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Upgrades</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Local BTS photographer / videographer</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D37" s="10">
+        <f>Assumptions!$B$5</f>
+        <v/>
+      </c>
+      <c r="E37" s="11">
+        <f>IF(H37="Y",C37*D37,0)</f>
+        <v/>
+      </c>
+      <c r="F37" s="12">
+        <f>E37/Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I37" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J37" s="10" t="inlineStr">
+        <is>
+          <t>Sponsor &amp; ministry assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Upgrades</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Legacy seed gift — Fondation Olivia Yacé</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="11">
+        <f>IF(H38="Y",C38*D38,0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="12">
+        <f>E38/Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I38" s="10" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="J38" s="10" t="inlineStr">
+        <is>
+          <t>Girls' school fees / goûter</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Travel (outside ground)</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Flights Accra → Abidjan</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D39" s="10">
+        <f>Assumptions!$B$3</f>
+        <v/>
+      </c>
+      <c r="E39" s="11">
+        <f>IF(H39="Y",C39*D39,0)</f>
+        <v/>
+      </c>
+      <c r="F39" s="12">
+        <f>E39/Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
           <t>Travel</t>
         </is>
       </c>
-      <c r="H36" s="13" t="inlineStr">
+      <c r="H39" s="13" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I36" s="10" t="inlineStr">
+      <c r="I39" s="10" t="inlineStr">
+        <is>
+          <t>In-kind: airline</t>
+        </is>
+      </c>
+      <c r="J39" s="10" t="inlineStr">
+        <is>
+          <t>May be on tour budget already</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Travel (outside ground)</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Flights Abidjan → Monrovia (Air Côte d'Ivoire)</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>280000</v>
+      </c>
+      <c r="D40" s="10">
+        <f>Assumptions!$B$3</f>
+        <v/>
+      </c>
+      <c r="E40" s="11">
+        <f>IF(H40="Y",C40*D40,0)</f>
+        <v/>
+      </c>
+      <c r="F40" s="12">
+        <f>E40/Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I40" s="10" t="inlineStr">
+        <is>
+          <t>In-kind: Air Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="J40" s="10" t="inlineStr">
+        <is>
+          <t>Check days for 22 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Travel (outside ground)</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>E-visas for non-ECOWAS crew</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D41" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="11">
+        <f>IF(H41="Y",C41*D41,0)</f>
+        <v/>
+      </c>
+      <c r="F41" s="12">
+        <f>E41/Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I41" s="10" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="J36" s="10" t="inlineStr">
+      <c r="J41" s="10" t="inlineStr">
         <is>
           <t>Ghanaian passports: none needed</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Ground costs — included lines (excl. travel)</t>
-        </is>
-      </c>
-      <c r="E38" s="14">
-        <f>SUMIFS(E3:E36,G3:G36,"&lt;&gt;Travel")</f>
-        <v/>
-      </c>
-      <c r="F38" s="15">
-        <f>E38/Assumptions!$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="E39" s="14">
-        <f>E38*Assumptions!$B$9</f>
-        <v/>
-      </c>
-      <c r="F39" s="15">
-        <f>E39/Assumptions!$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>AToure curation &amp; management fee</t>
-        </is>
-      </c>
-      <c r="E40" s="14">
-        <f>(E38+E39)*Assumptions!$B$10</f>
-        <v/>
-      </c>
-      <c r="F40" s="15">
-        <f>E40/Assumptions!$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL GROUND PROPOSITION</t>
-        </is>
-      </c>
-      <c r="E41" s="17">
-        <f>E38+E39+E40</f>
-        <v/>
-      </c>
-      <c r="F41" s="18">
-        <f>E41/Assumptions!$B$7</f>
-        <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>Travel lines included (reference, outside ground total)</t>
+          <t>Ground costs — included lines (excl. travel)</t>
         </is>
       </c>
       <c r="E43" s="14">
-        <f>SUMIFS(E3:E36,G3:G36,"Travel")</f>
+        <f>SUMIFS(E3:E41,G3:G41,"&lt;&gt;Travel")</f>
         <v/>
       </c>
       <c r="F43" s="15">
@@ -2322,9 +2452,69 @@
         <v/>
       </c>
     </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="E44" s="14">
+        <f>E43*Assumptions!$B$9</f>
+        <v/>
+      </c>
+      <c r="F44" s="15">
+        <f>E44/Assumptions!$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>AToure curation &amp; management fee</t>
+        </is>
+      </c>
+      <c r="E45" s="14">
+        <f>(E43+E44)*Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="F45" s="15">
+        <f>E45/Assumptions!$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL GROUND PROPOSITION</t>
+        </is>
+      </c>
+      <c r="E46" s="17">
+        <f>E43+E44+E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="18">
+        <f>E46/Assumptions!$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Travel lines included (reference, outside ground total)</t>
+        </is>
+      </c>
+      <c r="E48" s="14">
+        <f>SUMIFS(E3:E41,G3:G41,"Travel")</f>
+        <v/>
+      </c>
+      <c r="F48" s="15">
+        <f>E48/Assumptions!$B$7</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2377,10 +2567,10 @@
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>13554475</v>
+        <v>15540525</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>23990</v>
+        <v>27505</v>
       </c>
     </row>
     <row r="4">
@@ -2390,10 +2580,10 @@
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>16590475</v>
+        <v>18829525</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>29364</v>
+        <v>33327</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Budget v0.3 matching the deck itinerary (3 nights, relay kitchen, cocoa village)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsKwZ4mhRTGki8ZCbBAtxZ
</commit_message>
<xml_diff>
--- a/03-budget/ground-budget.xlsx
+++ b/03-budget/ground-budget.xlsx
@@ -534,11 +534,11 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nights of 18–21 Oct (arrive the evening before); depart 22 Oct to Monrovia</t>
+          <t>Nights of 19, 20, 21 Oct; depart 22 Oct to Monrovia</t>
         </is>
       </c>
     </row>
@@ -564,11 +564,11 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18 Oct airport pick-up through 22 Oct airport drop</t>
+          <t>19 Oct airport pick-up through 22 Oct airport drop</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -661,7 +661,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chef Abbys × Côte d'Ivoire · 19–21 Oct 2026 · Ground budget v0.2 (pre-quote estimate)</t>
+          <t>Chef Abbys × Côte d'Ivoire · 19–21 Oct 2026 · Ground budget v0.3 (pre-quote estimate)</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Airport protocol welcome + fast-track (arrival &amp; departure)</t>
+          <t>VIP airport welcome + fast-track (arrival &amp; departure)</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
@@ -754,7 +754,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>In-kind: ministry protocol</t>
+          <t>In-kind: Ministry of Tourism protocol</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>L'Avenue Hôtel (or equivalent), single rooms</t>
+          <t>Hotel 4–5★, single rooms</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
@@ -890,11 +890,7 @@
           <t>In-kind: telco</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Orange / MTN / Moov</t>
-        </is>
-      </c>
+      <c r="J6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -990,11 +986,11 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Fuel &amp; tolls supplement — Grand-Bassam run</t>
+          <t>Fuel &amp; tolls — cocoa village run</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>1</v>
@@ -1065,11 +1061,7 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
+      <c r="J10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1160,16 +1152,16 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · The lagoon</t>
+          <t>Day 1 · Snack time</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Attiéké entrepreneur — workshop honorarium</t>
+          <t>Goûter ingredients &amp; kit (~40 children)</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>300000</v>
+        <v>250000</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>1</v>
@@ -1194,24 +1186,24 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Sponsor</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Women-led brand, to identify</t>
+          <t>With Fondation Olivia Yacé</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · The lagoon</t>
+          <t>Day 1 · Snack time</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Lagoon beach location, set &amp; access</t>
+          <t>Burners, gas, aprons, hygiene</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
@@ -1243,25 +1235,21 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>Site to confirm</t>
-        </is>
-      </c>
+      <c r="J14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · The lagoon</t>
+          <t>Day 1 · Snack time</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Garba ingredients &amp; tasting</t>
+          <t>Child-safeguarding officer + consent forms</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>60000</v>
+        <v>100000</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>
@@ -1294,19 +1282,20 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · Snack time</t>
+          <t>Day 1 · Allocodrome</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Goûter ingredients &amp; kit (~40 children)</t>
+          <t>Tables, food &amp; drinks (party + ~6 guests)</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>1</v>
+        <v>20000</v>
+      </c>
+      <c r="D16" s="6">
+        <f>Assumptions!$B$3+6</f>
+        <v/>
       </c>
       <c r="E16" s="7">
         <f>IF(H16="Y",C16*D16,0)</f>
@@ -1331,25 +1320,21 @@
           <t>Sponsor</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>With Fondation Olivia Yacé</t>
-        </is>
-      </c>
+      <c r="J16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · Snack time</t>
+          <t>Day 1 · Allocodrome</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Burners, gas, aprons, hygiene</t>
+          <t>Jiaan Wu — co-host fee [TBC]</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>150000</v>
+        <v>300000</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>1</v>
@@ -1374,7 +1359,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Paid / exposure swap</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr"/>
@@ -1382,16 +1367,16 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · Snack time</t>
+          <t>Day 2 · Record day</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Child-safeguarding officer + consent forms</t>
+          <t>Zeinab Bancé — appearance fee [TBC]</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>100000</v>
+        <v>500000</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>1</v>
@@ -1419,25 +1404,21 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>Non-negotiable</t>
-        </is>
-      </c>
+      <c r="J18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · Maquis night</t>
+          <t>Day 2 · Record day</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Reserved space + live band</t>
+          <t>Speed duel set: mortars, timer, ingredients</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>350000</v>
+        <v>200000</v>
       </c>
       <c r="D19" s="6" t="n">
         <v>1</v>
@@ -1462,7 +1443,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr"/>
@@ -1470,20 +1451,19 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · Maquis night</t>
+          <t>Day 2 · Record day</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Food &amp; drinks (party + ~6 guests)</t>
+          <t>Relay kitchen — 1,000 plates</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D20" s="6">
-        <f>Assumptions!$B$3+6</f>
-        <v/>
+        <v>1500</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>1000</v>
       </c>
       <c r="E20" s="7">
         <f>IF(H20="Y",C20*D20,0)</f>
@@ -1508,21 +1488,25 @@
           <t>Sponsor</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>Food brand / FMCG</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Day 1 · Maquis night</t>
+          <t>Day 2 · Record day</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Jiaan Wu — co-host fee [TBC]</t>
+          <t>Relay kitchen — venue, tent, stoves, Treichville</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>300000</v>
+        <v>600000</v>
       </c>
       <c r="D21" s="6" t="n">
         <v>1</v>
@@ -1547,31 +1531,27 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Paid / exposure swap</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>Placeholder until quoted</t>
-        </is>
-      </c>
+          <t>In-kind: venue</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · Grand-Bassam</t>
+          <t>Day 2 · Record day</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Zeinab Bancé — foutou workshop fee</t>
+          <t>Servers &amp; volunteers (×10)</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>500000</v>
+        <v>15000</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E22" s="7">
         <f>IF(H22="Y",C22*D22,0)</f>
@@ -1596,25 +1576,21 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>Placeholder until quoted</t>
-        </is>
-      </c>
+      <c r="J22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · Grand-Bassam</t>
+          <t>Day 3 · Cocoa &amp; queens</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Lagoon-side garden location</t>
+          <t>Cocoa village — community contribution &amp; protocol</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>200000</v>
+        <v>300000</v>
       </c>
       <c r="D23" s="6" t="n">
         <v>1</v>
@@ -1639,7 +1615,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>In-kind: venue</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr"/>
@@ -1647,16 +1623,16 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · Grand-Bassam</t>
+          <t>Day 3 · Cocoa &amp; queens</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Ingredients, mortar, artisan crockery</t>
+          <t>Bean-to-bar workshop, Axel’s lab</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>150000</v>
+        <v>500000</v>
       </c>
       <c r="D24" s="6" t="n">
         <v>1</v>
@@ -1681,7 +1657,7 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>In-kind / co-brand</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr"/>
@@ -1689,16 +1665,16 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Day 2 · Grand-Bassam</t>
+          <t>Day 3 · Cocoa &amp; queens</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Heritage-quarter guide</t>
+          <t>Maison Mandjou atelier</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>50000</v>
+        <v>400000</v>
       </c>
       <c r="D25" s="6" t="n">
         <v>1</v>
@@ -1723,7 +1699,7 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>In-kind: Ministry of Culture</t>
+          <t>In-kind / co-brand</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr"/>
@@ -1731,19 +1707,20 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · Cocoa &amp; zaouli</t>
+          <t>Day 3 · Cocoa &amp; queens</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Maison Mandjou atelier (Ahoua Touré)</t>
+          <t>Closing dinner (party + ~10 guests)</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>400000</v>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>50000</v>
+      </c>
+      <c r="D26" s="6">
+        <f>Assumptions!$B$3+10</f>
+        <v/>
       </c>
       <c r="E26" s="7">
         <f>IF(H26="Y",C26*D26,0)</f>
@@ -1765,24 +1742,28 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>In-kind / co-brand</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr"/>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>Ministries, partners</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · Cocoa &amp; zaouli</t>
+          <t>Day 3 · Cocoa &amp; queens</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Bean-to-bar demo — partner chocolatier</t>
+          <t>Courtesy gifts</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>300000</v>
+        <v>100000</v>
       </c>
       <c r="D27" s="6" t="n">
         <v>1</v>
@@ -1807,31 +1788,27 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>In-kind / co-brand</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>e.g. Le Chocolatier Ivoirien</t>
-        </is>
-      </c>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · Cocoa &amp; zaouli</t>
+          <t>Production support</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Gouro zaouli troupe + musicians at KAVA</t>
+          <t>Licensed drone operator + ANAC authorisation</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="7">
         <f>IF(H28="Y",C28*D28,0)</f>
@@ -1853,27 +1830,32 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>In-kind: Ministry of Culture</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr"/>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>Days 2 &amp; 3</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Day 3 · Cocoa &amp; zaouli</t>
+          <t>Production support</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Customary gifts &amp; drinks — troupe</t>
+          <t>Welcome kit — pagne, AToure merch</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>1</v>
+        <v>25000</v>
+      </c>
+      <c r="D29" s="6">
+        <f>Assumptions!$B$3</f>
+        <v/>
       </c>
       <c r="E29" s="7">
         <f>IF(H29="Y",C29*D29,0)</f>
@@ -1901,199 +1883,192 @@
       <c r="J29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Day 3 · Closing table</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Closing dinner (party + ~10 guests)</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D30" s="6">
-        <f>Assumptions!$B$3+10</f>
-        <v/>
-      </c>
-      <c r="E30" s="7">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Upgrades</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Sponsored term of goûter for the school</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="11">
         <f>IF(H30="Y",C30*D30,0)</f>
         <v/>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="12">
         <f>E30/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
         <is>
           <t>Sponsor</t>
         </is>
       </c>
-      <c r="J30" s="6" t="inlineStr">
-        <is>
-          <t>Ministers, Olivia, chefs</t>
-        </is>
-      </c>
+      <c r="J30" s="10" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>Day 3 · Closing table</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Courtesy gifts (ministries, foundation)</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="7">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Upgrades</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Local BTS photographer / videographer</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D31" s="10">
+        <f>Assumptions!$B$5</f>
+        <v/>
+      </c>
+      <c r="E31" s="11">
         <f>IF(H31="Y",C31*D31,0)</f>
         <v/>
       </c>
-      <c r="F31" s="8">
+      <c r="F31" s="12">
         <f>E31/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr"/>
+      <c r="J31" s="10" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>Production support</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Licensed drone operator + ANAC authorisation</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>350000</v>
-      </c>
-      <c r="D32" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" s="7">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Travel (outside ground)</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Flights Accra → Abidjan</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D32" s="10">
+        <f>Assumptions!$B$3</f>
+        <v/>
+      </c>
+      <c r="E32" s="11">
         <f>IF(H32="Y",C32*D32,0)</f>
         <v/>
       </c>
-      <c r="F32" s="8">
+      <c r="F32" s="12">
         <f>E32/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>Days 1 &amp; 2</t>
-        </is>
-      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>In-kind: airline</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>Production support</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Welcome kit — pagne, AToure merch</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D33" s="6">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Travel (outside ground)</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Flights Abidjan → Monrovia (Air Côte d'Ivoire)</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>280000</v>
+      </c>
+      <c r="D33" s="10">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="11">
         <f>IF(H33="Y",C33*D33,0)</f>
         <v/>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="12">
         <f>E33/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="inlineStr"/>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>In-kind: Air Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="J33" s="10" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Upgrades</t>
+          <t>Travel (outside ground)</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>CASOF × Abidjan masterclass (20–30 young cooks)</t>
+          <t>E-visas for non-ECOWAS crew</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>300000</v>
+        <v>50000</v>
       </c>
       <c r="D34" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34" s="11">
         <f>IF(H34="Y",C34*D34,0)</f>
@@ -2105,7 +2080,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr">
@@ -2115,406 +2090,89 @@
       </c>
       <c r="I34" s="10" t="inlineStr">
         <is>
-          <t>Sponsor</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="J34" s="10" t="inlineStr"/>
     </row>
-    <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Cocoa farm visit (half day)</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D35" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="11">
-        <f>IF(H35="Y",C35*D35,0)</f>
-        <v/>
-      </c>
-      <c r="F35" s="12">
-        <f>E35/Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="G35" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>In-kind: Conseil Café-Cacao</t>
-        </is>
-      </c>
-      <c r="J35" s="10" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Sunset pinasse on the Ébrié lagoon</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="n">
-        <v>400000</v>
-      </c>
-      <c r="D36" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="11">
-        <f>IF(H36="Y",C36*D36,0)</f>
-        <v/>
-      </c>
-      <c r="F36" s="12">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ground costs — included lines (excl. travel)</t>
+        </is>
+      </c>
+      <c r="E36" s="14">
+        <f>SUMIFS(E3:E34,G3:G34,"&lt;&gt;Travel")</f>
+        <v/>
+      </c>
+      <c r="F36" s="15">
         <f>E36/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G36" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H36" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I36" s="10" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
-      <c r="J36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Local BTS photographer / videographer</t>
-        </is>
-      </c>
-      <c r="C37" s="11" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D37" s="10">
-        <f>Assumptions!$B$5</f>
-        <v/>
-      </c>
-      <c r="E37" s="11">
-        <f>IF(H37="Y",C37*D37,0)</f>
-        <v/>
-      </c>
-      <c r="F37" s="12">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="E37" s="14">
+        <f>E36*Assumptions!$B$9</f>
+        <v/>
+      </c>
+      <c r="F37" s="15">
         <f>E37/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G37" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I37" s="10" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="J37" s="10" t="inlineStr">
-        <is>
-          <t>Sponsor &amp; ministry assets</t>
-        </is>
-      </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>Upgrades</t>
-        </is>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Legacy seed gift — Fondation Olivia Yacé</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="D38" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="11">
-        <f>IF(H38="Y",C38*D38,0)</f>
-        <v/>
-      </c>
-      <c r="F38" s="12">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>AToure curation &amp; management fee</t>
+        </is>
+      </c>
+      <c r="E38" s="14">
+        <f>(E36+E37)*Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="F38" s="15">
         <f>E38/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G38" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H38" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I38" s="10" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
-      <c r="J38" s="10" t="inlineStr">
-        <is>
-          <t>Girls' school fees / goûter</t>
-        </is>
-      </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>Travel (outside ground)</t>
-        </is>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Flights Accra → Abidjan</t>
-        </is>
-      </c>
-      <c r="C39" s="11" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D39" s="10">
-        <f>Assumptions!$B$3</f>
-        <v/>
-      </c>
-      <c r="E39" s="11">
-        <f>IF(H39="Y",C39*D39,0)</f>
-        <v/>
-      </c>
-      <c r="F39" s="12">
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL GROUND PROPOSITION</t>
+        </is>
+      </c>
+      <c r="E39" s="17">
+        <f>E36+E37+E38</f>
+        <v/>
+      </c>
+      <c r="F39" s="18">
         <f>E39/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G39" s="10" t="inlineStr">
-        <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="H39" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I39" s="10" t="inlineStr">
-        <is>
-          <t>In-kind: airline</t>
-        </is>
-      </c>
-      <c r="J39" s="10" t="inlineStr">
-        <is>
-          <t>May be on tour budget already</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>Travel (outside ground)</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Flights Abidjan → Monrovia (Air Côte d'Ivoire)</t>
-        </is>
-      </c>
-      <c r="C40" s="11" t="n">
-        <v>280000</v>
-      </c>
-      <c r="D40" s="10">
-        <f>Assumptions!$B$3</f>
-        <v/>
-      </c>
-      <c r="E40" s="11">
-        <f>IF(H40="Y",C40*D40,0)</f>
-        <v/>
-      </c>
-      <c r="F40" s="12">
-        <f>E40/Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="G40" s="10" t="inlineStr">
-        <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="H40" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I40" s="10" t="inlineStr">
-        <is>
-          <t>In-kind: Air Côte d'Ivoire</t>
-        </is>
-      </c>
-      <c r="J40" s="10" t="inlineStr">
-        <is>
-          <t>Check days for 22 Oct</t>
-        </is>
-      </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Travel (outside ground)</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>E-visas for non-ECOWAS crew</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D41" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E41" s="11">
-        <f>IF(H41="Y",C41*D41,0)</f>
-        <v/>
-      </c>
-      <c r="F41" s="12">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Travel lines included (reference, outside ground total)</t>
+        </is>
+      </c>
+      <c r="E41" s="14">
+        <f>SUMIFS(E3:E34,G3:G34,"Travel")</f>
+        <v/>
+      </c>
+      <c r="F41" s="15">
         <f>E41/Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="G41" s="10" t="inlineStr">
-        <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="H41" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I41" s="10" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="J41" s="10" t="inlineStr">
-        <is>
-          <t>Ghanaian passports: none needed</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Ground costs — included lines (excl. travel)</t>
-        </is>
-      </c>
-      <c r="E43" s="14">
-        <f>SUMIFS(E3:E41,G3:G41,"&lt;&gt;Travel")</f>
-        <v/>
-      </c>
-      <c r="F43" s="15">
-        <f>E43/Assumptions!$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="E44" s="14">
-        <f>E43*Assumptions!$B$9</f>
-        <v/>
-      </c>
-      <c r="F44" s="15">
-        <f>E44/Assumptions!$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>AToure curation &amp; management fee</t>
-        </is>
-      </c>
-      <c r="E45" s="14">
-        <f>(E43+E44)*Assumptions!$B$10</f>
-        <v/>
-      </c>
-      <c r="F45" s="15">
-        <f>E45/Assumptions!$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL GROUND PROPOSITION</t>
-        </is>
-      </c>
-      <c r="E46" s="17">
-        <f>E43+E44+E45</f>
-        <v/>
-      </c>
-      <c r="F46" s="18">
-        <f>E46/Assumptions!$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Travel lines included (reference, outside ground total)</t>
-        </is>
-      </c>
-      <c r="E48" s="14">
-        <f>SUMIFS(E3:E41,G3:G41,"Travel")</f>
-        <v/>
-      </c>
-      <c r="F48" s="15">
-        <f>E48/Assumptions!$B$7</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2567,10 +2225,10 @@
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>15540525</v>
+        <v>15325475</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>27505</v>
+        <v>27125</v>
       </c>
     </row>
     <row r="4">
@@ -2580,10 +2238,10 @@
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>18829525</v>
+        <v>17349475</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>33327</v>
+        <v>30707</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Budget: add logistics-only scenario (stay, transport, ground team)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsKwZ4mhRTGki8ZCbBAtxZ
</commit_message>
<xml_diff>
--- a/03-budget/ground-budget.xlsx
+++ b/03-budget/ground-budget.xlsx
@@ -2186,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2234,26 +2234,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Core + all upgrades</t>
+          <t>Logistics only (stay, transport, ground team)</t>
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>17349475</v>
+        <v>6546375</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>30707</v>
+        <v>11587</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Core + all upgrades</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>17349475</v>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>30707</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Travel lines (if we must fund)</t>
         </is>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B6" s="14" t="n">
         <v>2980000</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C6" s="15" t="n">
         <v>5274</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Budget: security at 30k/officer/day, drop interpreter and meals from logistics, note who we will ask
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsKwZ4mhRTGki8ZCbBAtxZ
</commit_message>
<xml_diff>
--- a/03-budget/ground-budget.xlsx
+++ b/03-budget/ground-budget.xlsx
@@ -754,7 +754,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>In-kind: Ministry of Tourism protocol</t>
+          <t>Request: Ministry of Culture</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr"/>
@@ -807,47 +807,51 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Arrival &amp; stay</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Per diems — meals outside programme</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="11" t="n">
         <v>25000</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="10">
         <f>Assumptions!$B$3*Assumptions!$B$4</f>
         <v/>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="11">
         <f>IF(H5="Y",C5*D5,0)</f>
         <v/>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="12">
         <f>E5/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>Not in logistics budget</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -930,7 +934,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>In-kind: mobility partner</t>
+          <t>Request: Ghana High Commission / ministries</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr"/>
@@ -1021,47 +1025,51 @@
       <c r="J9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Ground team</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Bilingual fixer / on-camera interpreter (FR↔EN)</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="11" t="n">
         <v>80000</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="10">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="11">
         <f>IF(H10="Y",C10*D10,0)</f>
         <v/>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="12">
         <f>E10/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr"/>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>Not needed per Baba</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1071,11 +1079,11 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Protocol &amp; security officers (×2)</t>
+          <t>Security officers (×2)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="D11" s="6">
         <f>2*Assumptions!$B$5</f>
@@ -1104,50 +1112,54 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>30k per person per day</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Ground team</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Runner / production assistant</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="11" t="n">
         <v>25000</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="10">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="11">
         <f>IF(H12="Y",C12*D12,0)</f>
         <v/>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="12">
         <f>E12/Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr"/>
+      <c r="J12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2225,10 +2237,10 @@
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>15325475</v>
+        <v>14205950</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>27125</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="4">
@@ -2238,10 +2250,10 @@
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>6546375</v>
+        <v>5426850</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>11587</v>
+        <v>9605</v>
       </c>
     </row>
     <row r="5">
@@ -2251,10 +2263,10 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>17349475</v>
+        <v>17197675</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>30707</v>
+        <v>30438</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Budget: Sofitel quote (4 twin rooms, £2,800) and $200 airport welcome
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsKwZ4mhRTGki8ZCbBAtxZ
</commit_message>
<xml_diff>
--- a/03-budget/ground-budget.xlsx
+++ b/03-budget/ground-budget.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -545,88 +545,103 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Programme days</t>
+          <t>Hotel rooms</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>19–21 Oct</t>
+          <t>Twin rooms; Booking.com search 19–22 Oct, 4 rooms</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vehicle days</t>
+          <t>Programme days</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>19 Oct airport pick-up through 22 Oct airport drop</t>
+          <t>19–21 Oct</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>XOF per USD</t>
+          <t>Vehicle days</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>565</v>
+        <v>4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Check on the day</t>
+          <t>19 Oct airport pick-up through 22 Oct airport drop</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>XOF per EUR</t>
+          <t>XOF per USD</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>655.957</v>
+        <v>565</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fixed peg</t>
+          <t>Check on the day</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>0.1</v>
+          <t>XOF per EUR</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>655.957</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>On ground costs</t>
+          <t>Fixed peg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>On ground costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>AToure curation &amp; management fee</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B11" s="4" t="n">
         <v>0.15</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>PLACEHOLDER — Baba to set</t>
         </is>
@@ -729,7 +744,7 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>200000</v>
+        <v>56500</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>2</v>
@@ -739,7 +754,7 @@
         <v/>
       </c>
       <c r="F3" s="8">
-        <f>E3/Assumptions!$B$7</f>
+        <f>E3/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -767,14 +782,14 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Hotel 4–5★, single rooms</t>
+          <t>Sofitel Abidjan Hôtel Ivoire, twin rooms</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>150000</v>
+        <v>178500</v>
       </c>
       <c r="D4" s="6">
-        <f>Assumptions!$B$3*Assumptions!$B$4</f>
+        <f>Assumptions!$B$5*Assumptions!$B$4</f>
         <v/>
       </c>
       <c r="E4" s="7">
@@ -782,7 +797,7 @@
         <v/>
       </c>
       <c r="F4" s="8">
-        <f>E4/Assumptions!$B$7</f>
+        <f>E4/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -797,12 +812,12 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>In-kind: hotel partner</t>
+          <t>Request: Ministry of Tourism / hotel sponsor</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Rate to quote</t>
+          <t>Booking.com £2,800 incl. tax for 4 rooms × 3 nights, at £1 ≈ 765 XOF</t>
         </is>
       </c>
     </row>
@@ -829,7 +844,7 @@
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>E5/Assumptions!$B$7</f>
+        <f>E5/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -876,7 +891,7 @@
         <v/>
       </c>
       <c r="F6" s="8">
-        <f>E6/Assumptions!$B$7</f>
+        <f>E6/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -911,7 +926,7 @@
         <v>100000</v>
       </c>
       <c r="D7" s="6">
-        <f>Assumptions!$B$6</f>
+        <f>Assumptions!$B$7</f>
         <v/>
       </c>
       <c r="E7" s="7">
@@ -919,7 +934,7 @@
         <v/>
       </c>
       <c r="F7" s="8">
-        <f>E7/Assumptions!$B$7</f>
+        <f>E7/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -954,7 +969,7 @@
         <v>110000</v>
       </c>
       <c r="D8" s="6">
-        <f>Assumptions!$B$6</f>
+        <f>Assumptions!$B$7</f>
         <v/>
       </c>
       <c r="E8" s="7">
@@ -962,7 +977,7 @@
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>E8/Assumptions!$B$7</f>
+        <f>E8/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -1004,7 +1019,7 @@
         <v/>
       </c>
       <c r="F9" s="8">
-        <f>E9/Assumptions!$B$7</f>
+        <f>E9/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1039,7 +1054,7 @@
         <v>80000</v>
       </c>
       <c r="D10" s="10">
-        <f>Assumptions!$B$5</f>
+        <f>Assumptions!$B$6</f>
         <v/>
       </c>
       <c r="E10" s="11">
@@ -1047,7 +1062,7 @@
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>E10/Assumptions!$B$7</f>
+        <f>E10/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1086,7 +1101,7 @@
         <v>30000</v>
       </c>
       <c r="D11" s="6">
-        <f>2*Assumptions!$B$5</f>
+        <f>2*Assumptions!$B$6</f>
         <v/>
       </c>
       <c r="E11" s="7">
@@ -1094,7 +1109,7 @@
         <v/>
       </c>
       <c r="F11" s="8">
-        <f>E11/Assumptions!$B$7</f>
+        <f>E11/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1133,7 +1148,7 @@
         <v>25000</v>
       </c>
       <c r="D12" s="10">
-        <f>Assumptions!$B$5</f>
+        <f>Assumptions!$B$6</f>
         <v/>
       </c>
       <c r="E12" s="11">
@@ -1141,7 +1156,7 @@
         <v/>
       </c>
       <c r="F12" s="12">
-        <f>E12/Assumptions!$B$7</f>
+        <f>E12/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -1183,7 +1198,7 @@
         <v/>
       </c>
       <c r="F13" s="8">
-        <f>E13/Assumptions!$B$7</f>
+        <f>E13/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1229,7 +1244,7 @@
         <v/>
       </c>
       <c r="F14" s="8">
-        <f>E14/Assumptions!$B$7</f>
+        <f>E14/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1271,7 +1286,7 @@
         <v/>
       </c>
       <c r="F15" s="8">
-        <f>E15/Assumptions!$B$7</f>
+        <f>E15/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1314,7 +1329,7 @@
         <v/>
       </c>
       <c r="F16" s="8">
-        <f>E16/Assumptions!$B$7</f>
+        <f>E16/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1356,7 +1371,7 @@
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>E17/Assumptions!$B$7</f>
+        <f>E17/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1398,7 +1413,7 @@
         <v/>
       </c>
       <c r="F18" s="8">
-        <f>E18/Assumptions!$B$7</f>
+        <f>E18/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1440,7 +1455,7 @@
         <v/>
       </c>
       <c r="F19" s="8">
-        <f>E19/Assumptions!$B$7</f>
+        <f>E19/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1482,7 +1497,7 @@
         <v/>
       </c>
       <c r="F20" s="8">
-        <f>E20/Assumptions!$B$7</f>
+        <f>E20/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1528,7 +1543,7 @@
         <v/>
       </c>
       <c r="F21" s="8">
-        <f>E21/Assumptions!$B$7</f>
+        <f>E21/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1570,7 +1585,7 @@
         <v/>
       </c>
       <c r="F22" s="8">
-        <f>E22/Assumptions!$B$7</f>
+        <f>E22/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1612,7 +1627,7 @@
         <v/>
       </c>
       <c r="F23" s="8">
-        <f>E23/Assumptions!$B$7</f>
+        <f>E23/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1654,7 +1669,7 @@
         <v/>
       </c>
       <c r="F24" s="8">
-        <f>E24/Assumptions!$B$7</f>
+        <f>E24/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1696,7 +1711,7 @@
         <v/>
       </c>
       <c r="F25" s="8">
-        <f>E25/Assumptions!$B$7</f>
+        <f>E25/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1739,7 +1754,7 @@
         <v/>
       </c>
       <c r="F26" s="8">
-        <f>E26/Assumptions!$B$7</f>
+        <f>E26/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -1785,7 +1800,7 @@
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>E27/Assumptions!$B$7</f>
+        <f>E27/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -1827,7 +1842,7 @@
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>E28/Assumptions!$B$7</f>
+        <f>E28/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -1874,7 +1889,7 @@
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>E29/Assumptions!$B$7</f>
+        <f>E29/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -1916,7 +1931,7 @@
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>E30/Assumptions!$B$7</f>
+        <f>E30/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G30" s="10" t="inlineStr">
@@ -1951,7 +1966,7 @@
         <v>200000</v>
       </c>
       <c r="D31" s="10">
-        <f>Assumptions!$B$5</f>
+        <f>Assumptions!$B$6</f>
         <v/>
       </c>
       <c r="E31" s="11">
@@ -1959,7 +1974,7 @@
         <v/>
       </c>
       <c r="F31" s="12">
-        <f>E31/Assumptions!$B$7</f>
+        <f>E31/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G31" s="10" t="inlineStr">
@@ -2002,7 +2017,7 @@
         <v/>
       </c>
       <c r="F32" s="12">
-        <f>E32/Assumptions!$B$7</f>
+        <f>E32/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G32" s="10" t="inlineStr">
@@ -2045,7 +2060,7 @@
         <v/>
       </c>
       <c r="F33" s="12">
-        <f>E33/Assumptions!$B$7</f>
+        <f>E33/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G33" s="10" t="inlineStr">
@@ -2087,7 +2102,7 @@
         <v/>
       </c>
       <c r="F34" s="12">
-        <f>E34/Assumptions!$B$7</f>
+        <f>E34/Assumptions!$B$8</f>
         <v/>
       </c>
       <c r="G34" s="10" t="inlineStr">
@@ -2118,7 +2133,7 @@
         <v/>
       </c>
       <c r="F36" s="15">
-        <f>E36/Assumptions!$B$7</f>
+        <f>E36/Assumptions!$B$8</f>
         <v/>
       </c>
     </row>
@@ -2129,11 +2144,11 @@
         </is>
       </c>
       <c r="E37" s="14">
-        <f>E36*Assumptions!$B$9</f>
+        <f>E36*Assumptions!$B$10</f>
         <v/>
       </c>
       <c r="F37" s="15">
-        <f>E37/Assumptions!$B$7</f>
+        <f>E37/Assumptions!$B$8</f>
         <v/>
       </c>
     </row>
@@ -2144,11 +2159,11 @@
         </is>
       </c>
       <c r="E38" s="14">
-        <f>(E36+E37)*Assumptions!$B$10</f>
+        <f>(E36+E37)*Assumptions!$B$11</f>
         <v/>
       </c>
       <c r="F38" s="15">
-        <f>E38/Assumptions!$B$7</f>
+        <f>E38/Assumptions!$B$8</f>
         <v/>
       </c>
     </row>
@@ -2163,7 +2178,7 @@
         <v/>
       </c>
       <c r="F39" s="18">
-        <f>E39/Assumptions!$B$7</f>
+        <f>E39/Assumptions!$B$8</f>
         <v/>
       </c>
     </row>
@@ -2178,7 +2193,7 @@
         <v/>
       </c>
       <c r="F41" s="15">
-        <f>E41/Assumptions!$B$7</f>
+        <f>E41/Assumptions!$B$8</f>
         <v/>
       </c>
     </row>
@@ -2237,10 +2252,10 @@
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>14205950</v>
+        <v>13137025</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>25143</v>
+        <v>23251</v>
       </c>
     </row>
     <row r="4">
@@ -2250,10 +2265,10 @@
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>5426850</v>
+        <v>4357925</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>9605</v>
+        <v>7713</v>
       </c>
     </row>
     <row r="5">
@@ -2263,10 +2278,10 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>17197675</v>
+        <v>16128750</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>30438</v>
+        <v>28546</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Budget: remove AToure fee (not yet discussed); logistics total now $6,707
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsKwZ4mhRTGki8ZCbBAtxZ
</commit_message>
<xml_diff>
--- a/03-budget/ground-budget.xlsx
+++ b/03-budget/ground-budget.xlsx
@@ -639,11 +639,11 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — Baba to set</t>
+          <t>Not yet discussed with the client — left at 0</t>
         </is>
       </c>
     </row>
@@ -2252,10 +2252,10 @@
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>13137025</v>
+        <v>11423500</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>23251</v>
+        <v>20219</v>
       </c>
     </row>
     <row r="4">
@@ -2265,10 +2265,10 @@
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>4357925</v>
+        <v>3789500</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>7713</v>
+        <v>6707</v>
       </c>
     </row>
     <row r="5">
@@ -2278,10 +2278,10 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>16128750</v>
+        <v>14025000</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>28546</v>
+        <v>24823</v>
       </c>
     </row>
     <row r="6">

</xml_diff>